<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-06-02 02:58:27
</commit_message>
<xml_diff>
--- a/attendance_reports/Y2_B2526_GIT_&_Liver_session_analysis.xlsx
+++ b/attendance_reports/Y2_B2526_GIT_&_Liver_session_analysis.xlsx
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -842,7 +842,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8">
@@ -945,7 +945,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>27.6%</t>
+          <t>20.7%</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>34.1%</t>
+          <t>35.8%</t>
         </is>
       </c>
     </row>
@@ -1287,22 +1287,22 @@
         <v>29</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="Q15" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
-          <t>27.6%</t>
+          <t>20.7%</t>
         </is>
       </c>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>34.1%</t>
+          <t>35.8%</t>
         </is>
       </c>
     </row>
@@ -1350,49 +1350,45 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>Year 2</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>PARASITOLOGY</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>03/12/2025</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>08:00:00</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H17" s="5" t="inlineStr">
-        <is>
-          <t>80/251</t>
-        </is>
-      </c>
-      <c r="I17" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="G17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>0/251</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -1573,49 +1569,45 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>Year 2</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>PARASITOLOGY SGD/POS</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>03/12/2025</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>10:00:00</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H21" s="5" t="inlineStr">
-        <is>
-          <t>66/251</t>
-        </is>
-      </c>
-      <c r="I21" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="G21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>0/251</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">

</xml_diff>